<commit_message>
Inventorying donor site entries.
</commit_message>
<xml_diff>
--- a/source_data/donor_site_codes_annotated.xlsx
+++ b/source_data/donor_site_codes_annotated.xlsx
@@ -8,19 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/91aba14b6835b0ae/Work-current/Restoration_Storymap/2026_02_update/home_mbp/source_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C0922787-CA06-6443-B9CF-5C7CFEA4D369}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="58" documentId="8_{C0922787-CA06-6443-B9CF-5C7CFEA4D369}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{02721528-34DA-BF44-BB4C-03AAB4E1A3A2}"/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="720" windowWidth="28040" windowHeight="21160" xr2:uid="{4C48A302-F022-D04B-B3AC-943BB65EF98A}"/>
+    <workbookView xWindow="340" yWindow="700" windowWidth="28040" windowHeight="21160" activeTab="1" xr2:uid="{4C48A302-F022-D04B-B3AC-943BB65EF98A}"/>
   </bookViews>
   <sheets>
     <sheet name="donor_site_codes" sheetId="1" r:id="rId1"/>
+    <sheet name="crosswalk" sheetId="5" r:id="rId2"/>
+    <sheet name="gps_pts_donor_sites" sheetId="3" r:id="rId3"/>
+    <sheet name="donor_site_sheet_sites" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="60">
   <si>
     <t>donor_site_name</t>
   </si>
@@ -185,13 +188,28 @@
   </si>
   <si>
     <t>vicinity</t>
+  </si>
+  <si>
+    <t>donor_site_names</t>
+  </si>
+  <si>
+    <t>Elwha Delta</t>
+  </si>
+  <si>
+    <t>Cutts Island sandspit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">donor sirte sheet </t>
+  </si>
+  <si>
+    <t>no coords</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -326,8 +344,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="34">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -510,6 +535,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -674,9 +711,11 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1287,4 +1326,890 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D8E437D-CD60-6E49-8B52-3258BDBC6B45}">
+  <dimension ref="A2:H27"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="7" max="7" width="18.1640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B2" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C2" t="s">
+        <v>58</v>
+      </c>
+      <c r="G2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>3</v>
+      </c>
+      <c r="F4">
+        <v>2</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" t="s">
+        <v>5</v>
+      </c>
+      <c r="F5">
+        <v>3</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" t="s">
+        <v>57</v>
+      </c>
+      <c r="F6">
+        <v>4</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>7</v>
+      </c>
+      <c r="B7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" t="s">
+        <v>10</v>
+      </c>
+      <c r="F7">
+        <v>5</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>8</v>
+      </c>
+      <c r="B8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8">
+        <v>6</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9">
+        <v>7</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H9" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>10</v>
+      </c>
+      <c r="B10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" t="s">
+        <v>16</v>
+      </c>
+      <c r="F10">
+        <v>8</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H10" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>11</v>
+      </c>
+      <c r="B11" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="F11">
+        <v>9</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>12</v>
+      </c>
+      <c r="B12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F12">
+        <v>10</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>13</v>
+      </c>
+      <c r="B13" t="s">
+        <v>22</v>
+      </c>
+      <c r="C13" t="s">
+        <v>23</v>
+      </c>
+      <c r="F13">
+        <v>11</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>14</v>
+      </c>
+      <c r="B14" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" t="s">
+        <v>25</v>
+      </c>
+      <c r="F14">
+        <v>12</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A15">
+        <v>17</v>
+      </c>
+      <c r="B15" t="s">
+        <v>27</v>
+      </c>
+      <c r="C15" t="s">
+        <v>27</v>
+      </c>
+      <c r="F15">
+        <v>13</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A16">
+        <v>18</v>
+      </c>
+      <c r="B16" t="s">
+        <v>29</v>
+      </c>
+      <c r="C16" t="s">
+        <v>29</v>
+      </c>
+      <c r="F16">
+        <v>14</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A17">
+        <v>19</v>
+      </c>
+      <c r="B17" t="s">
+        <v>31</v>
+      </c>
+      <c r="C17" t="s">
+        <v>31</v>
+      </c>
+      <c r="F17">
+        <v>15</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A18">
+        <v>20</v>
+      </c>
+      <c r="B18" t="s">
+        <v>33</v>
+      </c>
+      <c r="C18" t="s">
+        <v>33</v>
+      </c>
+      <c r="F18">
+        <v>16</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A19">
+        <v>21</v>
+      </c>
+      <c r="B19" t="s">
+        <v>35</v>
+      </c>
+      <c r="C19" t="s">
+        <v>35</v>
+      </c>
+      <c r="F19">
+        <v>17</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A20">
+        <v>22</v>
+      </c>
+      <c r="B20" t="s">
+        <v>37</v>
+      </c>
+      <c r="C20" t="s">
+        <v>37</v>
+      </c>
+      <c r="F20">
+        <v>18</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A21">
+        <v>23</v>
+      </c>
+      <c r="B21" t="s">
+        <v>39</v>
+      </c>
+      <c r="C21" t="s">
+        <v>39</v>
+      </c>
+      <c r="D21" t="s">
+        <v>50</v>
+      </c>
+      <c r="F21">
+        <v>19</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A22">
+        <v>24</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="F22">
+        <v>20</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="H22" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A23">
+        <v>25</v>
+      </c>
+      <c r="B23" t="s">
+        <v>43</v>
+      </c>
+      <c r="C23" t="s">
+        <v>43</v>
+      </c>
+      <c r="F23">
+        <v>21</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A24">
+        <v>26</v>
+      </c>
+      <c r="B24" t="s">
+        <v>45</v>
+      </c>
+      <c r="C24" t="s">
+        <v>45</v>
+      </c>
+      <c r="F24">
+        <v>22</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B25" t="s">
+        <v>47</v>
+      </c>
+      <c r="C25" t="s">
+        <v>47</v>
+      </c>
+      <c r="F25">
+        <v>23</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A26">
+        <v>27</v>
+      </c>
+      <c r="B26" t="s">
+        <v>49</v>
+      </c>
+      <c r="C26" t="s">
+        <v>49</v>
+      </c>
+      <c r="D26" t="s">
+        <v>50</v>
+      </c>
+      <c r="F26">
+        <v>24</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A27">
+        <v>28</v>
+      </c>
+      <c r="B27" t="s">
+        <v>52</v>
+      </c>
+      <c r="C27" t="s">
+        <v>52</v>
+      </c>
+    </row>
+  </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="G3:G26">
+    <sortCondition ref="G3:G26"/>
+  </sortState>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A88FC2B-2CDC-2C43-A39D-4940EF36868B}">
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="27" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B1" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>5</v>
+      </c>
+      <c r="B5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>7</v>
+      </c>
+      <c r="B6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>8</v>
+      </c>
+      <c r="B7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>9</v>
+      </c>
+      <c r="B8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>10</v>
+      </c>
+      <c r="B9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>11</v>
+      </c>
+      <c r="B10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>12</v>
+      </c>
+      <c r="B11" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>13</v>
+      </c>
+      <c r="B12" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>14</v>
+      </c>
+      <c r="B13" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>17</v>
+      </c>
+      <c r="B14" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A15">
+        <v>18</v>
+      </c>
+      <c r="B15" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A16">
+        <v>19</v>
+      </c>
+      <c r="B16" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A17">
+        <v>20</v>
+      </c>
+      <c r="B17" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A18">
+        <v>21</v>
+      </c>
+      <c r="B18" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A19">
+        <v>22</v>
+      </c>
+      <c r="B19" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A20">
+        <v>23</v>
+      </c>
+      <c r="B20" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A21">
+        <v>24</v>
+      </c>
+      <c r="B21" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A22">
+        <v>25</v>
+      </c>
+      <c r="B22" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A23">
+        <v>26</v>
+      </c>
+      <c r="B23" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B24" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A25">
+        <v>27</v>
+      </c>
+      <c r="B25" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A26">
+        <v>28</v>
+      </c>
+      <c r="B26" t="s">
+        <v>52</v>
+      </c>
+    </row>
+  </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B1:B26">
+    <sortCondition ref="B1:B26"/>
+  </sortState>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9EF4D5A-7EDE-2344-AAD7-3EC502BF808D}">
+  <dimension ref="A1:B25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="18.1640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Tracking down donor site issues.
</commit_message>
<xml_diff>
--- a/source_data/donor_site_codes_annotated.xlsx
+++ b/source_data/donor_site_codes_annotated.xlsx
@@ -1,195 +1,107 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/91aba14b6835b0ae/Work-current/Restoration_Storymap/2026_02_update/home_mbp/source_data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stateofwa-my.sharepoint.com/personal/peter_dowty_dnr_wa_gov/Documents/projects/seagrass_restoration_data_2026/source_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="58" documentId="8_{C0922787-CA06-6443-B9CF-5C7CFEA4D369}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{02721528-34DA-BF44-BB4C-03AAB4E1A3A2}"/>
+  <xr:revisionPtr revIDLastSave="62" documentId="8_{C0922787-CA06-6443-B9CF-5C7CFEA4D369}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{850DBB85-2514-407B-9B6D-BBF537897FDB}"/>
   <bookViews>
-    <workbookView xWindow="340" yWindow="700" windowWidth="28040" windowHeight="21160" activeTab="1" xr2:uid="{4C48A302-F022-D04B-B3AC-943BB65EF98A}"/>
+    <workbookView xWindow="2295" yWindow="90" windowWidth="26505" windowHeight="15390" xr2:uid="{4C48A302-F022-D04B-B3AC-943BB65EF98A}"/>
   </bookViews>
   <sheets>
-    <sheet name="donor_site_codes" sheetId="1" r:id="rId1"/>
-    <sheet name="crosswalk" sheetId="5" r:id="rId2"/>
-    <sheet name="gps_pts_donor_sites" sheetId="3" r:id="rId3"/>
-    <sheet name="donor_site_sheet_sites" sheetId="4" r:id="rId4"/>
+    <sheet name="crosswalk" sheetId="5" r:id="rId1"/>
+    <sheet name="gps_pts_donor_sites" sheetId="3" r:id="rId2"/>
+    <sheet name="donor_site_sheet_sites" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="60">
-  <si>
-    <t>donor_site_name</t>
-  </si>
-  <si>
-    <t>alt_donor_site_name</t>
-  </si>
-  <si>
-    <t>donor_site_code</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="33">
   <si>
     <t>Bell Point</t>
   </si>
   <si>
-    <t>BPT</t>
-  </si>
-  <si>
     <t>Creosote Point</t>
   </si>
   <si>
-    <t>CPT</t>
-  </si>
-  <si>
     <t>Cutts Island</t>
   </si>
   <si>
-    <t>Cutts Island sand spit</t>
-  </si>
-  <si>
-    <t>CTI</t>
-  </si>
-  <si>
     <t>Dumas Bay</t>
   </si>
   <si>
-    <t>DMB</t>
-  </si>
-  <si>
     <t>DuPont Wharf</t>
   </si>
   <si>
-    <t>DPW</t>
-  </si>
-  <si>
     <t>Fay Bainbridge</t>
   </si>
   <si>
-    <t>FYB</t>
-  </si>
-  <si>
     <t>Freshwater Bay</t>
   </si>
   <si>
-    <t>FWB</t>
-  </si>
-  <si>
     <t>Green Point</t>
   </si>
   <si>
-    <t>GPT</t>
-  </si>
-  <si>
     <t>Henry Island</t>
   </si>
   <si>
-    <t>HRI</t>
-  </si>
-  <si>
     <t>Ketron Island</t>
   </si>
   <si>
     <t>Ketron Island NW</t>
   </si>
   <si>
-    <t>KTI</t>
-  </si>
-  <si>
     <t>Mitchell Bay</t>
   </si>
   <si>
-    <t>MTB</t>
-  </si>
-  <si>
     <t>PNNL - MSL Tanks</t>
   </si>
   <si>
-    <t>PNT</t>
-  </si>
-  <si>
     <t>Point Julia</t>
   </si>
   <si>
-    <t>PTJ</t>
-  </si>
-  <si>
     <t>Quilcene Bay</t>
   </si>
   <si>
-    <t>QLB</t>
-  </si>
-  <si>
     <t>Rocky Bay</t>
   </si>
   <si>
-    <t>RKB</t>
-  </si>
-  <si>
     <t>Rocky Point</t>
   </si>
   <si>
-    <t>RPT</t>
-  </si>
-  <si>
     <t>Sandy Hook</t>
   </si>
   <si>
-    <t>SNH</t>
-  </si>
-  <si>
     <t>Sandy Point</t>
   </si>
   <si>
-    <t>SPT</t>
-  </si>
-  <si>
     <t>Shine Beach</t>
   </si>
   <si>
-    <t>SHB</t>
-  </si>
-  <si>
     <t>Ship Harbor</t>
   </si>
   <si>
-    <t>SHH</t>
-  </si>
-  <si>
     <t>Skagit Bay</t>
   </si>
   <si>
-    <t>SKB</t>
-  </si>
-  <si>
     <t>Stuart Island</t>
   </si>
   <si>
-    <t>STI</t>
-  </si>
-  <si>
     <t>Thompson Cove</t>
   </si>
   <si>
     <t>Anderson Island</t>
   </si>
   <si>
-    <t>THC</t>
-  </si>
-  <si>
     <t>Windy Bluff</t>
   </si>
   <si>
-    <t>WNB</t>
-  </si>
-  <si>
-    <t>vicinity</t>
-  </si>
-  <si>
     <t>donor_site_names</t>
   </si>
   <si>
@@ -199,10 +111,16 @@
     <t>Cutts Island sandspit</t>
   </si>
   <si>
-    <t xml:space="preserve">donor sirte sheet </t>
-  </si>
-  <si>
     <t>no coords</t>
+  </si>
+  <si>
+    <t xml:space="preserve">donor site sheet </t>
+  </si>
+  <si>
+    <t>(from gps pts)</t>
+  </si>
+  <si>
+    <t>(from Matrix donor sheet)</t>
   </si>
 </sst>
 </file>
@@ -772,6 +690,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1090,692 +1012,461 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C7439C9-8733-D746-964C-13BEA0C8AA9F}">
-  <dimension ref="A1:D25"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="20.5" customWidth="1"/>
-    <col min="2" max="2" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.6640625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>54</v>
-      </c>
-      <c r="B1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B7" t="s">
-        <v>14</v>
-      </c>
-      <c r="D7" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B8" t="s">
-        <v>16</v>
-      </c>
-      <c r="D8" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B9" t="s">
-        <v>18</v>
-      </c>
-      <c r="D9" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B10" t="s">
-        <v>20</v>
-      </c>
-      <c r="D10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="D11" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B12" t="s">
-        <v>25</v>
-      </c>
-      <c r="D12" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B13" t="s">
-        <v>27</v>
-      </c>
-      <c r="D13" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B14" t="s">
-        <v>29</v>
-      </c>
-      <c r="D14" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B15" t="s">
-        <v>31</v>
-      </c>
-      <c r="D15" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B16" t="s">
-        <v>33</v>
-      </c>
-      <c r="D16" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B17" t="s">
-        <v>35</v>
-      </c>
-      <c r="D17" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B18" t="s">
-        <v>37</v>
-      </c>
-      <c r="D18" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A19" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="C19" s="1"/>
-      <c r="D19" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B20" t="s">
-        <v>41</v>
-      </c>
-      <c r="D20" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B21" t="s">
-        <v>43</v>
-      </c>
-      <c r="D21" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B22" t="s">
-        <v>45</v>
-      </c>
-      <c r="D22" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B23" t="s">
-        <v>47</v>
-      </c>
-      <c r="D23" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A24" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="C24" s="1"/>
-      <c r="D24" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B25" t="s">
-        <v>52</v>
-      </c>
-      <c r="D25" t="s">
-        <v>53</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D8E437D-CD60-6E49-8B52-3258BDBC6B45}">
-  <dimension ref="A2:H27"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:H27"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="16.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="21" customWidth="1"/>
     <col min="4" max="4" width="15" customWidth="1"/>
-    <col min="7" max="7" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B2" s="2" t="s">
-        <v>55</v>
+        <v>26</v>
       </c>
       <c r="C2" t="s">
-        <v>58</v>
+        <v>30</v>
       </c>
       <c r="G2" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>50</v>
+        <v>24</v>
       </c>
       <c r="D3" t="s">
-        <v>50</v>
+        <v>24</v>
       </c>
       <c r="F3">
         <v>1</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C4" t="s">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F4">
         <v>2</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C5" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F5">
         <v>3</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C6" t="s">
-        <v>57</v>
+        <v>28</v>
       </c>
       <c r="F6">
         <v>4</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>7</v>
       </c>
       <c r="B7" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="C7" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="F7">
         <v>5</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="C8" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="F8">
         <v>6</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>9</v>
       </c>
       <c r="B9" t="s">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="C9" t="s">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="F9">
         <v>7</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="H9" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="C10" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="F10">
         <v>8</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="H10" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="C11" t="s">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="F11">
         <v>9</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="C12" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="F12">
         <v>10</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>13</v>
       </c>
       <c r="B13" t="s">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="C13" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="F13">
         <v>11</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>14</v>
       </c>
       <c r="B14" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="C14" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="F14">
         <v>12</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>17</v>
       </c>
       <c r="B15" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="C15" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="F15">
         <v>13</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>18</v>
       </c>
       <c r="B16" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="C16" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="F16">
         <v>14</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>19</v>
       </c>
       <c r="B17" t="s">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="C17" t="s">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="F17">
         <v>15</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>20</v>
       </c>
       <c r="B18" t="s">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="C18" t="s">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="F18">
         <v>16</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>21</v>
       </c>
       <c r="B19" t="s">
-        <v>35</v>
+        <v>16</v>
       </c>
       <c r="C19" t="s">
-        <v>35</v>
+        <v>16</v>
       </c>
       <c r="F19">
         <v>17</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>22</v>
       </c>
       <c r="B20" t="s">
-        <v>37</v>
+        <v>17</v>
       </c>
       <c r="C20" t="s">
-        <v>37</v>
+        <v>17</v>
       </c>
       <c r="F20">
         <v>18</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>23</v>
       </c>
       <c r="B21" t="s">
-        <v>39</v>
+        <v>18</v>
       </c>
       <c r="C21" t="s">
-        <v>39</v>
+        <v>18</v>
       </c>
       <c r="D21" t="s">
-        <v>50</v>
+        <v>24</v>
       </c>
       <c r="F21">
         <v>19</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>24</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>41</v>
+        <v>19</v>
       </c>
       <c r="F22">
         <v>20</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="H22" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>25</v>
       </c>
       <c r="B23" t="s">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="C23" t="s">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="F23">
         <v>21</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>26</v>
       </c>
       <c r="B24" t="s">
-        <v>45</v>
+        <v>21</v>
       </c>
       <c r="C24" t="s">
-        <v>45</v>
+        <v>21</v>
       </c>
       <c r="F24">
         <v>22</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
-        <v>47</v>
+        <v>22</v>
       </c>
       <c r="C25" t="s">
-        <v>47</v>
+        <v>22</v>
       </c>
       <c r="F25">
         <v>23</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>27</v>
       </c>
       <c r="B26" t="s">
-        <v>49</v>
+        <v>23</v>
       </c>
       <c r="C26" t="s">
-        <v>49</v>
+        <v>23</v>
       </c>
       <c r="D26" t="s">
-        <v>50</v>
+        <v>24</v>
       </c>
       <c r="F26">
         <v>24</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>28</v>
       </c>
       <c r="B27" t="s">
-        <v>52</v>
+        <v>25</v>
       </c>
       <c r="C27" t="s">
-        <v>52</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -1786,214 +1477,214 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A88FC2B-2CDC-2C43-A39D-4940EF36868B}">
   <dimension ref="A1:B26"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B1" s="2" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>7</v>
       </c>
       <c r="B6" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>9</v>
       </c>
       <c r="B8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>13</v>
       </c>
       <c r="B12" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>14</v>
       </c>
       <c r="B13" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>17</v>
       </c>
       <c r="B14" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>18</v>
       </c>
       <c r="B15" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>19</v>
       </c>
       <c r="B16" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>20</v>
       </c>
       <c r="B17" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>21</v>
       </c>
       <c r="B18" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>22</v>
       </c>
       <c r="B19" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>23</v>
       </c>
       <c r="B20" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>24</v>
       </c>
       <c r="B21" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>25</v>
       </c>
       <c r="B22" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>26</v>
       </c>
       <c r="B23" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>27</v>
       </c>
       <c r="B25" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>28</v>
       </c>
       <c r="B26" t="s">
-        <v>52</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -2004,212 +1695,218 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9EF4D5A-7EDE-2344-AAD7-3EC502BF808D}">
   <dimension ref="A1:B25"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{11d0e217-264e-400a-8ba0-57dcc127d72d}" enabled="0" method="" siteId="{11d0e217-264e-400a-8ba0-57dcc127d72d}" removed="1"/>
+</clbl:labelList>
 </file>
</xml_diff>